<commit_message>
Update SW cache version to forcefully invalidate old UI layout cache
</commit_message>
<xml_diff>
--- a/Tubex_Aug26.xlsx
+++ b/Tubex_Aug26.xlsx
@@ -3927,7 +3927,7 @@
       <c r="G3" s="258"/>
       <c r="H3" s="263">
         <f ca="1">TODAY()-1</f>
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="I3" s="256"/>
       <c r="J3" s="256"/>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="C5" s="220">
         <f ca="1">TODAY()-1</f>
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="D5" s="114" t="s">
         <v>3</v>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="C7" s="221">
         <f ca="1">TODAY()-1</f>
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="D7" s="121" t="s">
         <v>11</v>
@@ -8951,7 +8951,7 @@
       </c>
       <c r="H1" s="136">
         <f ca="1">TODAY()</f>
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="I1" s="10"/>
       <c r="J1" s="11"/>
@@ -50901,7 +50901,7 @@
       </c>
       <c r="J1" s="63">
         <f ca="1">TODAY()</f>
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="64" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -51213,7 +51213,7 @@
       <c r="I12" s="67"/>
       <c r="J12" s="63">
         <f ca="1">TODAY()</f>
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix July PET production: accurately extract PF Machine Mustard Oil records (94,340 units) in customer report and archive
</commit_message>
<xml_diff>
--- a/Tubex_Aug26.xlsx
+++ b/Tubex_Aug26.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Alpha\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Alpha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_601DF1DA98759B46B83E03B9E04FAE33B3906977" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D346C11B-C7AC-40BE-865B-0EFEE6D789E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,8 +44,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4230" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4234" uniqueCount="620">
   <si>
     <t>TUBEX  — August 2026 Month to Date Report</t>
   </si>
@@ -1904,6 +1926,9 @@
   <si>
     <t>19</t>
   </si>
+  <si>
+    <t>Caps &amp; Slug Shortage</t>
+  </si>
 </sst>
 </file>
 
@@ -3520,12 +3545,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="31" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="31" fillId="3" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3535,19 +3573,6 @@
     <xf numFmtId="0" fontId="37" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="31" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3961,7 +3986,7 @@
     <col min="1" max="1" width="1.5703125" style="105" customWidth="1"/>
     <col min="2" max="2" width="7" style="105" customWidth="1"/>
     <col min="3" max="3" width="32.7109375" style="105" customWidth="1"/>
-    <col min="4" max="4" width="38.7109375" style="105" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" style="105" customWidth="1"/>
     <col min="5" max="5" width="8.85546875" style="103" customWidth="1"/>
     <col min="6" max="6" width="9.140625" style="105" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="12.140625" style="106" customWidth="1"/>
@@ -4009,22 +4034,22 @@
     </row>
     <row r="2" spans="1:29" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="102"/>
-      <c r="B2" s="269" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="262"/>
-      <c r="D2" s="262"/>
-      <c r="E2" s="263"/>
-      <c r="F2" s="262"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="262"/>
-      <c r="I2" s="262"/>
-      <c r="J2" s="262"/>
-      <c r="K2" s="262"/>
-      <c r="L2" s="262"/>
-      <c r="M2" s="262"/>
-      <c r="N2" s="262"/>
-      <c r="O2" s="262"/>
+      <c r="B2" s="263" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="264"/>
+      <c r="D2" s="264"/>
+      <c r="E2" s="265"/>
+      <c r="F2" s="264"/>
+      <c r="G2" s="266"/>
+      <c r="H2" s="264"/>
+      <c r="I2" s="264"/>
+      <c r="J2" s="264"/>
+      <c r="K2" s="264"/>
+      <c r="L2" s="264"/>
+      <c r="M2" s="264"/>
+      <c r="N2" s="264"/>
+      <c r="O2" s="264"/>
       <c r="P2" s="102"/>
       <c r="Q2" s="102"/>
       <c r="R2" s="102"/>
@@ -4042,25 +4067,25 @@
     </row>
     <row r="3" spans="1:29" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="102"/>
-      <c r="B3" s="261" t="s">
+      <c r="B3" s="269" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="262"/>
-      <c r="D3" s="262"/>
-      <c r="E3" s="263"/>
-      <c r="F3" s="262"/>
-      <c r="G3" s="264"/>
-      <c r="H3" s="266">
+      <c r="C3" s="264"/>
+      <c r="D3" s="264"/>
+      <c r="E3" s="265"/>
+      <c r="F3" s="264"/>
+      <c r="G3" s="266"/>
+      <c r="H3" s="271">
         <f>MAX(Production_Log!$A$3:$A$8961)</f>
-        <v>46248</v>
-      </c>
-      <c r="I3" s="262"/>
-      <c r="J3" s="262"/>
-      <c r="K3" s="262"/>
-      <c r="L3" s="262"/>
-      <c r="M3" s="262"/>
-      <c r="N3" s="262"/>
-      <c r="O3" s="262"/>
+        <v>46250</v>
+      </c>
+      <c r="I3" s="264"/>
+      <c r="J3" s="264"/>
+      <c r="K3" s="264"/>
+      <c r="L3" s="264"/>
+      <c r="M3" s="264"/>
+      <c r="N3" s="264"/>
+      <c r="O3" s="264"/>
       <c r="P3" s="102"/>
       <c r="Q3" s="102"/>
       <c r="R3" s="102"/>
@@ -4113,22 +4138,22 @@
       </c>
       <c r="C5" s="195">
         <f>MAX(Production_Log!$A$3:$A$8961)</f>
-        <v>46248</v>
+        <v>46250</v>
       </c>
       <c r="D5" s="107" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="107"/>
       <c r="F5" s="108"/>
-      <c r="G5" s="268" t="s">
+      <c r="G5" s="267" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="262"/>
+      <c r="H5" s="264"/>
       <c r="I5" s="109"/>
-      <c r="J5" s="268" t="s">
+      <c r="J5" s="267" t="s">
         <v>5</v>
       </c>
-      <c r="K5" s="262"/>
+      <c r="K5" s="264"/>
       <c r="L5" s="136"/>
       <c r="M5" s="110" t="s">
         <v>6</v>
@@ -4152,28 +4177,28 @@
     </row>
     <row r="6" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="102"/>
-      <c r="B6" s="265">
+      <c r="B6" s="270">
         <f>SUMPRODUCT((Production_Log!$A$3:$A$8961=MAX(Production_Log!$A$3:$A$8961))*(LEFT(Production_Log!$B$3:$B$8961,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8961)))*Production_Log!$H$3:$H$8961)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="262"/>
+      <c r="C6" s="264"/>
       <c r="D6" s="111">
         <f>SUMIF($B$11:$B$66,"TUBE",$H$11:$H$66)</f>
         <v>212464</v>
       </c>
-      <c r="E6" s="265"/>
-      <c r="F6" s="262"/>
+      <c r="E6" s="270"/>
+      <c r="F6" s="264"/>
       <c r="G6" s="112">
         <f t="array" ref="G6">IFERROR(SUMPRODUCT((Production_Log!$F$3:$F$8961&lt;&gt;0)*(LEFT(Production_Log!$B$3:$B$8961,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8961)))*Production_Log!$I$3:$I$8961)/SUMPRODUCT((Production_Log!$F$3:$F$8961&lt;&gt;0)*(LEFT(Production_Log!$B$3:$B$8961,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8961)))*(Production_Log!$H$3:$H$8961+Production_Log!$I$3:$I$8961)),"-")</f>
         <v>2.0605345404593103E-2</v>
       </c>
       <c r="H6" s="112"/>
       <c r="I6" s="109"/>
-      <c r="J6" s="265">
+      <c r="J6" s="270">
         <f>SUMIF($B$11:$B$66,"TUBE",$K$11:$K$66)</f>
         <v>164682</v>
       </c>
-      <c r="K6" s="262"/>
+      <c r="K6" s="264"/>
       <c r="L6" s="113"/>
       <c r="M6" s="137" t="s">
         <v>7</v>
@@ -4206,17 +4231,17 @@
       </c>
       <c r="C7" s="196">
         <f>MAX(Production_Log!$A$3:$A$8961)</f>
-        <v>46248</v>
+        <v>46250</v>
       </c>
       <c r="D7" s="114" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="114"/>
       <c r="F7" s="115"/>
-      <c r="G7" s="267" t="s">
+      <c r="G7" s="272" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="262"/>
+      <c r="H7" s="264"/>
       <c r="I7" s="116"/>
       <c r="J7" s="115" t="s">
         <v>5</v>
@@ -4252,28 +4277,28 @@
     </row>
     <row r="8" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="102"/>
-      <c r="B8" s="270">
+      <c r="B8" s="268">
         <f>SUMPRODUCT((Production_Log!$A$3:$A$8961=MAX(Production_Log!$A$3:$A$8961))*(Production_Log!$B$3:$B$8961="PF Machine")*Production_Log!$H$3:$H$8961)</f>
-        <v>8740</v>
-      </c>
-      <c r="C8" s="262"/>
+        <v>0</v>
+      </c>
+      <c r="C8" s="264"/>
       <c r="D8" s="117">
         <f>SUMIF($B$11:$B$66,"PET",$H$11:$H$66)</f>
         <v>60375</v>
       </c>
-      <c r="E8" s="270"/>
-      <c r="F8" s="262"/>
+      <c r="E8" s="268"/>
+      <c r="F8" s="264"/>
       <c r="G8" s="118">
         <f t="array" ref="G8">IFERROR(SUMPRODUCT((Production_Log!$B$3:$B$8961="PF Machine")*Production_Log!$I$3:$I$8961)/SUMPRODUCT((Production_Log!$B$3:$B$8961="PF Machine")*(Production_Log!$H$3:$H$8961+Production_Log!$I$3:$I$8961)),0)</f>
         <v>5.0483604623732012E-2</v>
       </c>
       <c r="H8" s="118"/>
       <c r="I8" s="116"/>
-      <c r="J8" s="270">
+      <c r="J8" s="268">
         <f>SUMIF($B$11:$B$66,"PET",$K$11:$K$66)</f>
         <v>31280</v>
       </c>
-      <c r="K8" s="262"/>
+      <c r="K8" s="264"/>
       <c r="L8" s="119"/>
       <c r="M8" s="123" t="str">
         <f>IFERROR(INDEX($S$9:$S$22,MATCH(LARGE($U$9:$U$22,2),$U$9:$U$22,0)),"")</f>
@@ -4304,19 +4329,19 @@
     </row>
     <row r="9" spans="1:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="102"/>
-      <c r="B9" s="271" t="s">
+      <c r="B9" s="261" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="272"/>
-      <c r="D9" s="272"/>
-      <c r="E9" s="272"/>
-      <c r="F9" s="272"/>
-      <c r="G9" s="272"/>
-      <c r="H9" s="272"/>
-      <c r="I9" s="272"/>
-      <c r="J9" s="272"/>
-      <c r="K9" s="272"/>
-      <c r="L9" s="272"/>
+      <c r="C9" s="262"/>
+      <c r="D9" s="262"/>
+      <c r="E9" s="262"/>
+      <c r="F9" s="262"/>
+      <c r="G9" s="262"/>
+      <c r="H9" s="262"/>
+      <c r="I9" s="262"/>
+      <c r="J9" s="262"/>
+      <c r="K9" s="262"/>
+      <c r="L9" s="262"/>
       <c r="M9" s="123" t="str">
         <f>IFERROR(INDEX($S$9:$S$22,MATCH(LARGE($U$9:$U$22,3),$U$9:$U$22,0)),"")</f>
         <v>Mechanical</v>
@@ -4790,17 +4815,17 @@
       <c r="G17" s="252">
         <v>701257</v>
       </c>
-      <c r="H17" s="253">
-        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F17)*Production_Log!$H$3:$H$8963)</f>
-        <v>60375</v>
+      <c r="H17" s="253" cm="1">
+        <f t="array" ref="H17">SUMPRODUCT((Production_Log!$F$3:$F$8963=F17)*Production_Log!$H$3:$H$8963)-13960</f>
+        <v>46415</v>
       </c>
       <c r="I17" s="252">
         <f>G17-H17</f>
-        <v>640882</v>
+        <v>654842</v>
       </c>
       <c r="J17" s="254">
         <f>IF(G17=0,"-",H17/G17)</f>
-        <v>8.6095397265196646E-2</v>
+        <v>6.6188287603546198E-2</v>
       </c>
       <c r="K17" s="253">
         <v>31280</v>
@@ -4855,16 +4880,15 @@
         <v>13960</v>
       </c>
       <c r="H18" s="253">
-        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F18)*Production_Log!$H$3:$H$8963)</f>
-        <v>0</v>
+        <v>13960</v>
       </c>
       <c r="I18" s="252">
         <f>G18-H18</f>
-        <v>13960</v>
+        <v>0</v>
       </c>
       <c r="J18" s="254">
         <f>IF(G18=0,"-",H18/G18)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="253"/>
       <c r="L18" s="255" t="s">
@@ -9062,8 +9086,8 @@
     <col min="6" max="6" width="16.5703125" style="4" customWidth="1"/>
     <col min="7" max="7" width="11.7109375" style="5" customWidth="1"/>
     <col min="8" max="8" width="17.5703125" style="4" customWidth="1"/>
-    <col min="9" max="9" width="15" style="3" customWidth="1"/>
-    <col min="10" max="10" width="46.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="45.42578125" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
     <col min="13" max="13" width="24" customWidth="1"/>
@@ -9083,7 +9107,7 @@
       </c>
       <c r="H1" s="129">
         <f ca="1">TODAY()</f>
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="I1" s="10"/>
       <c r="J1" s="11"/>
@@ -9163,7 +9187,9 @@
         <f>F3-G3</f>
         <v>107458</v>
       </c>
-      <c r="I3" s="205"/>
+      <c r="I3" s="205" t="s">
+        <v>619</v>
+      </c>
     </row>
     <row r="4" spans="1:19" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12"/>
@@ -9690,15 +9716,15 @@
       </c>
       <c r="F17" s="200">
         <f>IFERROR(INDEX(TableInventory[Store Balance],MATCH(A17,TableInventory[Item ID],0)),0)+IFERROR(INDEX(TableInventory[Work In Process],MATCH(A17,TableInventory[Item ID],0)),0)</f>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G17" s="199">
         <f t="shared" si="0"/>
-        <v>-885.63040000000001</v>
+        <v>-945.63040000000001</v>
       </c>
       <c r="H17" s="226">
         <f>IFERROR(IF(SUMPRODUCT((TableBOM[Item ID]=A17)*(TableBOM[Product ID]=$D$3)*($H$3&gt;0)*TableBOM[Per 1000 Units])=0,"-",ROUND(F17/(SUMPRODUCT((TableBOM[Item ID]=A17)*(TableBOM[Product ID]=$D$3)*($H$3&gt;0)*TableBOM[Per 1000 Units])/1000),0)),"-")</f>
-        <v>7500</v>
+        <v>0</v>
       </c>
       <c r="I17" s="201" t="str">
         <f t="shared" si="1"/>
@@ -9782,11 +9808,11 @@
       </c>
       <c r="F19" s="199">
         <f>IFERROR(INDEX(TableInventory[Store Balance],MATCH(A19,TableInventory[Item ID],0)),0)+IFERROR(INDEX(TableInventory[Work In Process],MATCH(A19,TableInventory[Item ID],0)),0)</f>
-        <v>444</v>
+        <v>425</v>
       </c>
       <c r="G19" s="199">
         <f t="shared" si="0"/>
-        <v>444</v>
+        <v>425</v>
       </c>
       <c r="H19" s="226" t="str">
         <f>IFERROR(IF(SUMPRODUCT((TableBOM[Item ID]=A19)*(TableBOM[Product ID]=$D$3)*($H$3&gt;0)*TableBOM[Per 1000 Units])=0,"-",ROUND(F19/(SUMPRODUCT((TableBOM[Item ID]=A19)*(TableBOM[Product ID]=$D$3)*($H$3&gt;0)*TableBOM[Per 1000 Units])/1000),0)),"-")</f>
@@ -11885,7 +11911,7 @@
         <v>427</v>
       </c>
       <c r="G71" s="199">
-        <f t="shared" ref="G71:G102" si="6">F71-E71</f>
+        <f t="shared" ref="G71:G88" si="6">F71-E71</f>
         <v>408.56020719999998</v>
       </c>
       <c r="H71" s="226">
@@ -12702,11 +12728,11 @@
       </c>
       <c r="G95" s="220">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$100,MATCH(MRP!D95,Tubex_Dashboard!$F$11:$F$100,0))</f>
-        <v>60375</v>
+        <v>46415</v>
       </c>
       <c r="H95" s="221">
         <f>F95-G95</f>
-        <v>640882</v>
+        <v>654842</v>
       </c>
       <c r="I95" s="192"/>
     </row>
@@ -12731,11 +12757,11 @@
       </c>
       <c r="G96" s="222">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$100,MATCH(MRP!D96,Tubex_Dashboard!$F$11:$F$100,0))</f>
-        <v>0</v>
+        <v>13960</v>
       </c>
       <c r="H96" s="223">
         <f>F96-G96</f>
-        <v>13960</v>
+        <v>0</v>
       </c>
       <c r="I96" s="192"/>
       <c r="J96" s="189"/>
@@ -15997,7 +16023,7 @@
         <v>50</v>
       </c>
       <c r="J67" s="234">
-        <f t="shared" ref="J67:J98" si="2">IFERROR(I67/(H67+I67),"")</f>
+        <f t="shared" ref="J67:J73" si="2">IFERROR(I67/(H67+I67),"")</f>
         <v>7.1942446043165471E-3</v>
       </c>
       <c r="K67" s="232"/>
@@ -16269,25 +16295,46 @@
       <c r="S73" s="232"/>
     </row>
     <row r="74" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="176"/>
-      <c r="B74" s="177"/>
-      <c r="C74" s="177"/>
-      <c r="D74" s="177"/>
-      <c r="E74" s="177"/>
-      <c r="F74" s="177"/>
-      <c r="G74" s="178"/>
-      <c r="H74" s="178"/>
-      <c r="I74" s="178"/>
-      <c r="J74" s="179"/>
-      <c r="K74" s="177"/>
-      <c r="L74" s="177"/>
-      <c r="M74" s="177"/>
-      <c r="N74" s="177"/>
-      <c r="O74" s="177"/>
-      <c r="P74" s="177"/>
-      <c r="Q74" s="177"/>
-      <c r="R74" s="177"/>
-      <c r="S74" s="177"/>
+      <c r="A74" s="231">
+        <v>46250</v>
+      </c>
+      <c r="B74" s="232" t="s">
+        <v>262</v>
+      </c>
+      <c r="C74" s="232" t="s">
+        <v>30</v>
+      </c>
+      <c r="D74" s="232" t="s">
+        <v>31</v>
+      </c>
+      <c r="E74" s="232">
+        <v>30</v>
+      </c>
+      <c r="F74" s="232">
+        <v>6206</v>
+      </c>
+      <c r="G74" s="233">
+        <v>0</v>
+      </c>
+      <c r="H74" s="233">
+        <v>0</v>
+      </c>
+      <c r="I74" s="233">
+        <v>0</v>
+      </c>
+      <c r="J74" s="234" t="str">
+        <f t="shared" ref="J74" si="3">IFERROR(I74/(H74+I74),"")</f>
+        <v/>
+      </c>
+      <c r="K74" s="232"/>
+      <c r="L74" s="232"/>
+      <c r="M74" s="232"/>
+      <c r="N74" s="232"/>
+      <c r="O74" s="232"/>
+      <c r="P74" s="232"/>
+      <c r="Q74" s="232"/>
+      <c r="R74" s="232"/>
+      <c r="S74" s="232"/>
     </row>
     <row r="75" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="176"/>
@@ -52383,19 +52430,19 @@
       <c r="A1" s="278" t="s">
         <v>333</v>
       </c>
-      <c r="B1" s="272"/>
-      <c r="C1" s="272"/>
-      <c r="D1" s="272"/>
-      <c r="E1" s="272"/>
-      <c r="F1" s="272"/>
-      <c r="G1" s="272"/>
-      <c r="H1" s="272"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
       <c r="I1" s="55" t="s">
         <v>114</v>
       </c>
       <c r="J1" s="56">
         <f ca="1">TODAY()</f>
-        <v>46251</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="57" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -52618,12 +52665,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I8" s="28">
-        <v>60</v>
-      </c>
+      <c r="I8" s="28"/>
       <c r="J8" s="157">
         <f>IFERROR(IF(AVERAGEIF(TableBOM[Item ID],A8,TableBOM[Per 1000 Units])=0,"-",ROUND((H8+I8)/(AVERAGEIF(TableBOM[Item ID],A8,TableBOM[Per 1000 Units])/1000),0)),"-")</f>
-        <v>7500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -52652,12 +52697,10 @@
         <f t="shared" si="0"/>
         <v>425</v>
       </c>
-      <c r="I9" s="28">
-        <v>19</v>
-      </c>
+      <c r="I9" s="28"/>
       <c r="J9" s="157">
         <f>IFERROR(IF(AVERAGEIF(TableBOM[Item ID],A9,TableBOM[Per 1000 Units])=0,"-",ROUND((H9+I9)/(AVERAGEIF(TableBOM[Item ID],A9,TableBOM[Per 1000 Units])/1000),0)),"-")</f>
-        <v>40872</v>
+        <v>39123</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -52709,7 +52752,7 @@
       <c r="I12" s="60"/>
       <c r="J12" s="56">
         <f ca="1">TODAY()</f>
-        <v>46251</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -55154,7 +55197,7 @@
         <v>0</v>
       </c>
       <c r="H78" s="145">
-        <f t="shared" ref="H78:H109" si="3">E78+F78-G78</f>
+        <f t="shared" ref="H78:H92" si="3">E78+F78-G78</f>
         <v>1</v>
       </c>
       <c r="I78" s="144"/>
@@ -62974,15 +63017,15 @@
     </sortState>
   </autoFilter>
   <mergeCells count="9">
+    <mergeCell ref="A92:K92"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A81:K81"/>
+    <mergeCell ref="A75:K75"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A23:K23"/>
     <mergeCell ref="A34:K34"/>
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A92:K92"/>
-    <mergeCell ref="A65:K65"/>
-    <mergeCell ref="A81:K81"/>
-    <mergeCell ref="A75:K75"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>